<commit_message>
update selections csv data
</commit_message>
<xml_diff>
--- a/public/files/csv/selections.xlsx
+++ b/public/files/csv/selections.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28925"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MOHCINE\Desktop\SIM APPS\selection\public\files\csv\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TRANS_AA\Desktop\selection\public\files\csv\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{077A6555-2885-4661-A0B1-1D4B4043DB99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="500"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
   <si>
     <t>TAN TAN</t>
   </si>
@@ -49,12 +48,6 @@
     <t>2°BRB</t>
   </si>
   <si>
-    <t>AL HOCEIMA</t>
-  </si>
-  <si>
-    <t>1°BIMAR</t>
-  </si>
-  <si>
     <t>OUARZAZATE</t>
   </si>
   <si>
@@ -140,12 +133,24 @@
   </si>
   <si>
     <t>1°BN</t>
+  </si>
+  <si>
+    <t>10°BLIR</t>
+  </si>
+  <si>
+    <t>FES</t>
+  </si>
+  <si>
+    <t>1°GT</t>
+  </si>
+  <si>
+    <t>AIN HARROUDA</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <fonts count="2">
     <font>
       <sz val="11"/>
@@ -198,9 +203,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -238,9 +243,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -275,7 +280,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -310,7 +315,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -483,8 +488,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B20"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:B21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.5703125" customWidth="1"/>
@@ -501,7 +506,7 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B2" t="s">
         <v>1</v>
@@ -533,122 +538,130 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
-        <v>10</v>
+        <v>38</v>
       </c>
       <c r="B6" t="s">
-        <v>9</v>
+        <v>39</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B7" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="1" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B8" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B9" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B10" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B11" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B12" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B13" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B14" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B15" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B16" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="1" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B17" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B18" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="19" spans="1:2">
       <c r="A19" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="20" spans="1:2">
       <c r="A20" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B20" t="s">
-        <v>28</v>
+        <v>26</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2">
+      <c r="A21" t="s">
+        <v>40</v>
+      </c>
+      <c r="B21" t="s">
+        <v>41</v>
       </c>
     </row>
   </sheetData>

</xml_diff>